<commit_message>
[feat] MatchScheduleUI 상대 목록 / 경기 요청 패널 로직
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/OrganizationData.xlsx
+++ b/JsonConverter/ExcelFiles/OrganizationData.xlsx
@@ -19,39 +19,42 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="11">
+<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="12">
   <x:si>
     <x:t>Id</x:t>
-  </x:si>
-  <x:si>
-    <x:t>프로토타입용 테스트 최초의 리그다</x:t>
   </x:si>
   <x:si>
     <x:t>fighter_02,fighter_03,fighter_04</x:t>
   </x:si>
   <x:si>
-    <x:t>Description</x:t>
+    <x:t>여기에 적는 순서에 따라 랭킹이 정해짐. (가장 앞: 챔피언, 그 뒤로부터 랭킹 1~10위 처럼)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>고유 ID</x:t>
+  </x:si>
+  <x:si>
+    <x:t>string</x:t>
+  </x:si>
+  <x:si>
+    <x:t>프로토 리그</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Name</x:t>
+  </x:si>
+  <x:si>
+    <x:t>org_01</x:t>
+  </x:si>
+  <x:si>
+    <x:t>(name)</x:t>
   </x:si>
   <x:si>
     <x:t>FighterIds</x:t>
   </x:si>
   <x:si>
-    <x:t>org_01</x:t>
+    <x:t>Description</x:t>
   </x:si>
   <x:si>
-    <x:t>string</x:t>
-  </x:si>
-  <x:si>
-    <x:t>고유 ID</x:t>
-  </x:si>
-  <x:si>
-    <x:t>프로토 리그</x:t>
-  </x:si>
-  <x:si>
-    <x:t>(name)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Name</x:t>
+    <x:t>프로토타입용 테스트 최초의 리그다</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -836,23 +839,26 @@
     <x:col min="13" max="16384" width="12.54296875" style="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" spans="1:1" ht="15.75" customHeight="1">
+    <x:row r="1" spans="1:4" ht="15.75" customHeight="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>7</x:v>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D1" s="1" t="s">
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:4" ht="13.199999999999999">
       <x:c r="A2" s="1" t="s">
-        <x:v>9</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="B2" s="1" t="s">
-        <x:v>6</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C2" s="1" t="s">
-        <x:v>6</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D2" s="1" t="s">
-        <x:v>6</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:4" s="7" customFormat="1" ht="15.75" customHeight="1">
@@ -860,27 +866,27 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="B3" s="2" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C3" s="2" t="s">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="C3" s="2" t="s">
-        <x:v>3</x:v>
-      </x:c>
       <x:c r="D3" s="7" t="s">
-        <x:v>4</x:v>
+        <x:v>9</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:6" ht="15.75" customHeight="1">
       <x:c r="A4" s="3" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B4" s="3" t="s">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="B4" s="3" t="s">
-        <x:v>8</x:v>
-      </x:c>
       <x:c r="C4" s="3" t="s">
-        <x:v>1</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="D4" s="1" t="s">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F4" s="4"/>
     </x:row>

</xml_diff>